<commit_message>
Updated JPN model - 2025-09-07 18:53
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_JPN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_JPN\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{61A75C8A-ED05-43FE-8EED-46AD54C89BB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0333D973-3AD1-4C5E-862A-EE6AB0BEEB7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8510,7 +8510,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B01A3603-82E8-4CCB-9837-5DC06401E1AD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59BB6B63-9FE2-4C14-AEDA-10280AF0B279}">
   <dimension ref="B9:N39"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -9668,7 +9668,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66469083-4509-472A-9E5C-51777F3BA1AD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1806B6C8-318D-4722-9539-20DEE482BFD9}">
   <dimension ref="B9:AB241"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -26428,7 +26428,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6738AAB2-9210-451B-B7AA-CB6AB124E09F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B31C9C49-846F-4E7E-A032-7B908616A2F4}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated JPN model - 2025-09-07 19:14
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_JPN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_JPN\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0333D973-3AD1-4C5E-862A-EE6AB0BEEB7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7F0E7737-7FAA-4CA1-B261-EA00A9EEDBBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8510,7 +8510,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59BB6B63-9FE2-4C14-AEDA-10280AF0B279}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5802F4D-0230-43F1-8FB1-6369D1D7D6E7}">
   <dimension ref="B9:N39"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -9668,7 +9668,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1806B6C8-318D-4722-9539-20DEE482BFD9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AF68027-24AC-4069-A67D-86189CAAA42E}">
   <dimension ref="B9:AB241"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -26428,7 +26428,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B31C9C49-846F-4E7E-A032-7B908616A2F4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05661A8E-2B62-49A2-AFE4-9CD86DE300CD}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated JPN model - 2025-09-13 01:23
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_JPN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_JPN\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1E0C5931-ABF5-4F8B-8A11-3855FAD91442}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D2E5345B-809C-4F8E-97B8-E4630896E948}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8514,7 +8514,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9EC5C238-B9CD-498D-9B65-95B6F65081B1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8AEC6E7F-5523-4A63-9A18-D8029A540311}">
   <dimension ref="B9:N39"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -9672,7 +9672,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BF41302-6226-408E-B251-2B31AB2C6A24}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3FEB1845-3FBC-4C1C-AB9B-3B997CF215DE}">
   <dimension ref="B9:AB241"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -26432,7 +26432,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD608A1B-7EA0-4B2B-AF5A-364DE8246974}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9879DE1-FCF7-4CE2-9382-1CFB4DFBCCD0}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated JPN model - 2025-09-13 08:58
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_JPN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_JPN\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D2E5345B-809C-4F8E-97B8-E4630896E948}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{003CD53D-E5F0-4CD8-88C0-26F11AC49688}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8514,7 +8514,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8AEC6E7F-5523-4A63-9A18-D8029A540311}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E800B49A-E3FF-4577-80E6-A1E193CB4054}">
   <dimension ref="B9:N39"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -9672,7 +9672,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3FEB1845-3FBC-4C1C-AB9B-3B997CF215DE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{552660D0-F3B0-4B75-8E5A-6A2659DE5450}">
   <dimension ref="B9:AB241"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -26432,7 +26432,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9879DE1-FCF7-4CE2-9382-1CFB4DFBCCD0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B12574F-B45B-47BD-B425-DF3552F569AE}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated JPN model - 2025-09-13 09:41
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_JPN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_JPN\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{003CD53D-E5F0-4CD8-88C0-26F11AC49688}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D4B87CD0-B586-4CDC-8D60-9334095BC048}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8514,7 +8514,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E800B49A-E3FF-4577-80E6-A1E193CB4054}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6254FE7-32D3-4851-91A6-3E96EFD356A7}">
   <dimension ref="B9:N39"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -9672,7 +9672,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{552660D0-F3B0-4B75-8E5A-6A2659DE5450}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5BB1278-07BE-47EA-B270-6EDCC15059BE}">
   <dimension ref="B9:AB241"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -26432,7 +26432,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B12574F-B45B-47BD-B425-DF3552F569AE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBFE0899-2434-4DB1-96B5-F9AA160147CC}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated JPN model - 2025-09-13 16:30
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_JPN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_JPN\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D4B87CD0-B586-4CDC-8D60-9334095BC048}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{47908D9E-3EAE-4837-89C8-8D8622919513}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8514,7 +8514,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6254FE7-32D3-4851-91A6-3E96EFD356A7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CE58A2C-AE11-47B2-A51A-46B1E60942E6}">
   <dimension ref="B9:N39"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -9672,7 +9672,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5BB1278-07BE-47EA-B270-6EDCC15059BE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8BC06A9-646E-45D1-B6D0-1F42C09DB17E}">
   <dimension ref="B9:AB241"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -26432,7 +26432,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBFE0899-2434-4DB1-96B5-F9AA160147CC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A5B9B7E-B9C6-44F2-BDC7-B87F30334D2F}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated JPN model - 2025-09-14 19:29
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_JPN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_JPN\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{47908D9E-3EAE-4837-89C8-8D8622919513}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{215F13A8-4738-469B-8E0D-9F5AFECE2582}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8514,7 +8514,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CE58A2C-AE11-47B2-A51A-46B1E60942E6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92D0186C-36BE-40AE-BCF9-F5DB73593165}">
   <dimension ref="B9:N39"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -9672,7 +9672,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8BC06A9-646E-45D1-B6D0-1F42C09DB17E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{457E2D50-91F6-43F2-B968-58D10D47613B}">
   <dimension ref="B9:AB241"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -26432,7 +26432,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A5B9B7E-B9C6-44F2-BDC7-B87F30334D2F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{615D0D19-041E-4FB2-9BA6-4EB3D6A88355}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated JPN model - 2025-09-23 09:03
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_JPN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_JPN\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{14313848-E9D6-4BEF-A978-E8EA90940790}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F278295E-CF87-4F90-9936-C887E3270015}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6399,7 +6399,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3F2387E-E909-4DDE-BD94-D2F7C728C49D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81B81187-24EB-42E5-ACB2-306A4A4B17F1}">
   <dimension ref="B9:M41"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -7537,7 +7537,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0A81C70-740E-44E3-AD4B-68DE7C43F594}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{509658F7-2092-4AA5-9FF6-39EE42C42E5D}">
   <dimension ref="B9:Z54"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -10192,7 +10192,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A14D618-2117-4EA9-AF99-D31E89019D0A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{857E82F3-DCCD-4BE9-99BE-185880BFC6FD}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>